<commit_message>
Updated the orchestrator and model selector
</commit_message>
<xml_diff>
--- a/artifacts/expense_tracker.xlsx
+++ b/artifacts/expense_tracker.xlsx
@@ -424,17 +424,17 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Description</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Category</t>
         </is>
       </c>
     </row>
@@ -450,11 +450,11 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Food</t>
+          <t>Weekly grocery shopping</t>
         </is>
       </c>
     </row>
@@ -466,15 +466,15 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Dinner at Restaurant</t>
+          <t>Transportation</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>45.99</v>
+        <v>60</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Entertainment</t>
+          <t>Bus fare to work</t>
         </is>
       </c>
     </row>
@@ -486,15 +486,15 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Gasoline</t>
+          <t>Entertainment</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>30.75</v>
+        <v>40</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Transportation</t>
+          <t>Movie night</t>
         </is>
       </c>
     </row>

</xml_diff>